<commit_message>
feat(wave4): complete and benchmark P0 vertical slices for 05-mini-quic, 04-columnar, 02-hnsw
</commit_message>
<xml_diff>
--- a/projects/02-hnsw-filtered-vector-index/spreadsheets/02_hnsw-filtered-vector-index_features.xlsx
+++ b/projects/02-hnsw-filtered-vector-index/spreadsheets/02_hnsw-filtered-vector-index_features.xlsx
@@ -726,7 +726,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -780,7 +780,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -834,7 +834,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -942,7 +942,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -996,7 +996,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -1158,7 +1158,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -1266,7 +1266,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1374,7 +1374,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -1428,7 +1428,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -1482,7 +1482,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
@@ -1536,7 +1536,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -1590,7 +1590,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
@@ -1644,7 +1644,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
@@ -1698,7 +1698,7 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
@@ -1860,7 +1860,7 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
@@ -1914,7 +1914,7 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
@@ -2022,7 +2022,7 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
@@ -2076,7 +2076,7 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
@@ -2130,7 +2130,7 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
@@ -2400,7 +2400,7 @@
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
@@ -2508,7 +2508,7 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
@@ -2562,7 +2562,7 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
@@ -2616,7 +2616,7 @@
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
@@ -2670,7 +2670,7 @@
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
@@ -2724,7 +2724,7 @@
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
@@ -2778,7 +2778,7 @@
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="M40" t="inlineStr">
@@ -2832,7 +2832,7 @@
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="M41" t="inlineStr">
@@ -2886,7 +2886,7 @@
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="M42" t="inlineStr">
@@ -3156,7 +3156,7 @@
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="M47" t="inlineStr">
@@ -3264,7 +3264,7 @@
       </c>
       <c r="L49" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="M49" t="inlineStr">
@@ -3318,7 +3318,7 @@
       </c>
       <c r="L50" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="M50" t="inlineStr">
@@ -3372,7 +3372,7 @@
       </c>
       <c r="L51" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="M51" t="inlineStr">
@@ -3480,7 +3480,7 @@
       </c>
       <c r="L53" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="M53" t="inlineStr">
@@ -3534,7 +3534,7 @@
       </c>
       <c r="L54" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="M54" t="inlineStr">
@@ -3588,7 +3588,7 @@
       </c>
       <c r="L55" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="M55" t="inlineStr">
@@ -3750,7 +3750,7 @@
       </c>
       <c r="L58" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="M58" t="inlineStr">
@@ -3804,7 +3804,7 @@
       </c>
       <c r="L59" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="M59" t="inlineStr">
@@ -3858,7 +3858,7 @@
       </c>
       <c r="L60" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="M60" t="inlineStr">
@@ -3912,7 +3912,7 @@
       </c>
       <c r="L61" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="M61" t="inlineStr">
@@ -3966,7 +3966,7 @@
       </c>
       <c r="L62" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="M62" t="inlineStr">
@@ -4074,7 +4074,7 @@
       </c>
       <c r="L64" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="M64" t="inlineStr">
@@ -4128,7 +4128,7 @@
       </c>
       <c r="L65" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="M65" t="inlineStr">
@@ -4182,7 +4182,7 @@
       </c>
       <c r="L66" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="M66" t="inlineStr">
@@ -4236,7 +4236,7 @@
       </c>
       <c r="L67" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="M67" t="inlineStr">
@@ -4290,7 +4290,7 @@
       </c>
       <c r="L68" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="M68" t="inlineStr">
@@ -4344,7 +4344,7 @@
       </c>
       <c r="L69" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="M69" t="inlineStr">
@@ -4398,7 +4398,7 @@
       </c>
       <c r="L70" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="M70" t="inlineStr">
@@ -4452,7 +4452,7 @@
       </c>
       <c r="L71" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="M71" t="inlineStr">
@@ -4614,7 +4614,7 @@
       </c>
       <c r="L74" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="M74" t="inlineStr">
@@ -4668,7 +4668,7 @@
       </c>
       <c r="L75" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="M75" t="inlineStr">
@@ -4722,7 +4722,7 @@
       </c>
       <c r="L76" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="M76" t="inlineStr">
@@ -4776,7 +4776,7 @@
       </c>
       <c r="L77" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="M77" t="inlineStr">
@@ -5046,7 +5046,7 @@
       </c>
       <c r="L82" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="M82" t="inlineStr">
@@ -5100,7 +5100,7 @@
       </c>
       <c r="L83" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="M83" t="inlineStr">
@@ -5154,7 +5154,7 @@
       </c>
       <c r="L84" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="M84" t="inlineStr">
@@ -5208,7 +5208,7 @@
       </c>
       <c r="L85" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="M85" t="inlineStr">
@@ -5262,7 +5262,7 @@
       </c>
       <c r="L86" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="M86" t="inlineStr">
@@ -5316,7 +5316,7 @@
       </c>
       <c r="L87" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="M87" t="inlineStr">
@@ -5424,7 +5424,7 @@
       </c>
       <c r="L89" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="M89" t="inlineStr">
@@ -5478,7 +5478,7 @@
       </c>
       <c r="L90" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="M90" t="inlineStr">
@@ -5532,7 +5532,7 @@
       </c>
       <c r="L91" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="M91" t="inlineStr">
@@ -5694,7 +5694,7 @@
       </c>
       <c r="L94" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="M94" t="inlineStr">
@@ -5748,7 +5748,7 @@
       </c>
       <c r="L95" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="M95" t="inlineStr">
@@ -5856,7 +5856,7 @@
       </c>
       <c r="L97" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="M97" t="inlineStr">
@@ -5910,7 +5910,7 @@
       </c>
       <c r="L98" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="M98" t="inlineStr">
@@ -5964,7 +5964,7 @@
       </c>
       <c r="L99" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="M99" t="inlineStr">
@@ -6018,7 +6018,7 @@
       </c>
       <c r="L100" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="M100" t="inlineStr">
@@ -8986,7 +8986,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -9031,7 +9031,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -9121,7 +9121,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -9166,7 +9166,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -9211,7 +9211,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -9256,7 +9256,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -9301,7 +9301,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -9497,7 +9497,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -9542,7 +9542,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -9632,7 +9632,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -9677,7 +9677,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -9812,7 +9812,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -9902,7 +9902,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -9992,7 +9992,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -10037,7 +10037,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -10082,7 +10082,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -10127,7 +10127,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -10172,7 +10172,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -10217,7 +10217,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -10352,7 +10352,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -10397,7 +10397,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -10442,7 +10442,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -10487,7 +10487,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -10532,7 +10532,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -10757,7 +10757,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -10847,7 +10847,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -10892,7 +10892,7 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -10937,7 +10937,7 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -10982,7 +10982,7 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -11027,7 +11027,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -11072,7 +11072,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -11117,7 +11117,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -11342,7 +11342,7 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -11387,7 +11387,7 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -11432,7 +11432,7 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -11522,7 +11522,7 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
@@ -11567,7 +11567,7 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
@@ -11702,7 +11702,7 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
@@ -11747,7 +11747,7 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
@@ -11792,7 +11792,7 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
@@ -11837,7 +11837,7 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
@@ -11882,7 +11882,7 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
@@ -11972,7 +11972,7 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
@@ -12017,7 +12017,7 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
@@ -12062,7 +12062,7 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
@@ -12107,7 +12107,7 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
@@ -12152,7 +12152,7 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
@@ -12197,7 +12197,7 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
@@ -12242,7 +12242,7 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
@@ -12287,7 +12287,7 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
@@ -12422,7 +12422,7 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
@@ -12467,7 +12467,7 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
@@ -12512,7 +12512,7 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
@@ -12737,7 +12737,7 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
@@ -12782,7 +12782,7 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
@@ -12827,7 +12827,7 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
@@ -12872,7 +12872,7 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
@@ -12917,7 +12917,7 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
@@ -12962,7 +12962,7 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
@@ -13052,7 +13052,7 @@
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
@@ -13097,7 +13097,7 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
@@ -13187,7 +13187,7 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
@@ -13232,7 +13232,7 @@
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="H85" t="inlineStr">
@@ -13277,7 +13277,7 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
@@ -15543,7 +15543,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -15694,7 +15694,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -15829,7 +15829,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">

</xml_diff>